<commit_message>
Add the refined-mesh check of the 10 s release
V2 on the 33.2 kJ, 500 mW/K case with a 10 s release, every mesh spacing
halved (297,057 nodes): the hottest-point crossing times move by at most
0.020 s (0.0001 s at 183.5 C) against the unrounded base run, the peak of
the hottest point by +1.49 K, and its location is unchanged. With this,
both releases of the headline case have both V2 checks; the note's check
line now covers them together.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JRQdFboVN1WcGEdwURaRN7
</commit_message>
<xml_diff>
--- a/results/pilot_b_results.xlsx
+++ b/results/pilot_b_results.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="181">
   <si>
     <t xml:space="preserve">Pilot B: two LG M50 cells, resolved against lumped neighbour. Repository github.com/siddharth161204-wq/m50-two-cell-pilot</t>
   </si>
@@ -420,6 +420,15 @@
   </si>
   <si>
     <t xml:space="preserve">V2 max energy, tau 10 s, 500 mW/K, time step halved (0.05 s) (against an unrounded base run): change in resolved mean peak (K)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V2 max energy, tau 10 s, 500 mW/K, mesh refined (297,057 nodes) (against an unrounded base run): largest change in a hottest-point crossing time (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V2 max energy, tau 10 s, 500 mW/K, mesh refined (297,057 nodes) (against an unrounded base run): change in resolved max peak (K)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V2 max energy, tau 10 s, 500 mW/K, mesh refined (297,057 nodes) (against an unrounded base run): change in resolved mean peak (K)</t>
   </si>
   <si>
     <t xml:space="preserve">V2 max energy, tau 30 s, 500 mW/K, time step halved (0.05 s) (against an unrounded base run): largest change in a hottest-point crossing time (s)</t>
@@ -7199,7 +7208,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -7291,7 +7300,7 @@
         <v>131</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.00327365881429564</v>
+        <v>0.0200216726846616</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7299,7 +7308,7 @@
         <v>132</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.0398145369898657</v>
+        <v>1.48897783640496</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7307,7 +7316,7 @@
         <v>133</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.00551631911679351</v>
+        <v>-0.305821865303415</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7315,7 +7324,7 @@
         <v>134</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.0847956586240528</v>
+        <v>0.00327365881429564</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7323,7 +7332,7 @@
         <v>135</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>1.41088468164253</v>
+        <v>0.0398145369898657</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7331,47 +7340,47 @@
         <v>136</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>-0.307861475483378</v>
+        <v>0.00551631911679351</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>138</v>
+      <c r="B17" s="2" t="n">
+        <v>0.0847956586240528</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B18" s="2" t="s">
         <v>138</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>1.41088468164253</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>0</v>
+        <v>-0.307861475483378</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B21" s="2" t="n">
-        <v>85.700699276118</v>
+      <c r="B21" s="2" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7379,7 +7388,7 @@
         <v>143</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>82.9629522175588</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7387,15 +7396,15 @@
         <v>144</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>96.718297592367</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B24" s="5" t="n">
-        <v>1.2E-011</v>
+      <c r="B24" s="2" t="n">
+        <v>85.700699276118</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7403,7 +7412,7 @@
         <v>146</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0.308102760535576</v>
+        <v>82.9629522175588</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7411,6 +7420,30 @@
         <v>147</v>
       </c>
       <c r="B26" s="2" t="n">
+        <v>96.718297592367</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1.2E-011</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>0.308102760535576</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B29" s="2" t="n">
         <v>0.169868364338555</v>
       </c>
     </row>
@@ -7451,7 +7484,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>8</v>
@@ -7463,37 +7496,37 @@
         <v>10</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>26</v>
@@ -7501,7 +7534,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>33222.9</v>
@@ -7551,7 +7584,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>33222.9</v>
@@ -7601,7 +7634,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>21495.3</v>
@@ -7631,7 +7664,7 @@
         <v>134.023204376743</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>152.8</v>
@@ -7651,7 +7684,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>33222.9</v>
@@ -7681,7 +7714,7 @@
         <v>153.92403509182</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>168.9</v>
@@ -7701,7 +7734,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>33222.9</v>
@@ -7751,7 +7784,7 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>8</v>
@@ -7763,27 +7796,27 @@
         <v>10</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>33222.9</v>
@@ -7815,7 +7848,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>21495.3</v>
@@ -7842,12 +7875,12 @@
         <v>22.9911075058746</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>33222.9</v>
@@ -7874,12 +7907,12 @@
         <v>23.9667529712611</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>21495.3</v>
@@ -7903,15 +7936,15 @@
         <v>0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>33222.9</v>
@@ -7935,15 +7968,15 @@
         <v>0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>33222.9</v>
@@ -7975,7 +8008,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>33222.9</v>
@@ -8002,12 +8035,12 @@
         <v>10.4706385650631</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>21495.3</v>
@@ -8034,7 +8067,7 @@
         <v>8.84197793287098</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>